<commit_message>
Add interactive upload flow, clickable quality issues, and derived-column provenance
- Upload screen now starts empty and walks through uploading the six
  source extracts with per-file progress; loaded-source detail opens in a
  full-width bottom panel instead of the cramped right drawer
- Data quality issues are clickable and reveal example rows pulled from
  the actual source data (generator now attaches per-issue examples)
- AutoMap screen lists every derived column with a plain-language meaning
  and the source files it is synthesized from
</commit_message>
<xml_diff>
--- a/Publications_Trials_Scientific_Activity.xlsx
+++ b/Publications_Trials_Scientific_Activity.xlsx
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>secondary prevention;stroke rehabilitation;ischemic stroke;telestroke</t>
+          <t>ischemic stroke;telestroke;stroke rehabilitation;secondary prevention</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>lipid management;antiplatelet therapy;secondary prevention;ischemic stroke;telestroke</t>
+          <t>ischemic stroke;telestroke;secondary prevention;lipid management;antiplatelet therapy</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>lipid management;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;secondary prevention;lipid management</t>
         </is>
       </c>
       <c r="I117" t="n">
@@ -8974,7 +8974,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>lipid management;secondary prevention;telestroke;ischemic stroke;atrial fibrillation</t>
+          <t>ischemic stroke;telestroke;secondary prevention;lipid management;atrial fibrillation</t>
         </is>
       </c>
       <c r="I152" t="n">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>endovascular thrombectomy;secondary prevention;ischemic stroke;telestroke;TIA</t>
+          <t>ischemic stroke;TIA;telestroke;secondary prevention;endovascular thrombectomy</t>
         </is>
       </c>
       <c r="I163" t="n">
@@ -19662,7 +19662,7 @@
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke;antiplatelet therapy</t>
+          <t>ischemic stroke;secondary prevention;antiplatelet therapy</t>
         </is>
       </c>
       <c r="I343" t="n">
@@ -22022,7 +22022,7 @@
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke;endovascular thrombectomy</t>
+          <t>ischemic stroke;secondary prevention;endovascular thrombectomy</t>
         </is>
       </c>
       <c r="I385" t="n">
@@ -23714,7 +23714,7 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke;telestroke;antiplatelet therapy</t>
+          <t>ischemic stroke;telestroke;secondary prevention;antiplatelet therapy</t>
         </is>
       </c>
       <c r="I416" t="n">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>telestroke;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;telestroke;secondary prevention</t>
         </is>
       </c>
       <c r="I443" t="n">
@@ -26094,7 +26094,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>cerebrovascular imaging;secondary prevention;TIA;ischemic stroke</t>
+          <t>ischemic stroke;secondary prevention;TIA;cerebrovascular imaging</t>
         </is>
       </c>
       <c r="I459" t="n">
@@ -27410,7 +27410,7 @@
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>antiplatelet therapy;secondary prevention;ischemic stroke;telestroke;atrial fibrillation</t>
+          <t>ischemic stroke;telestroke;secondary prevention;antiplatelet therapy;atrial fibrillation</t>
         </is>
       </c>
       <c r="I483" t="n">
@@ -27466,7 +27466,7 @@
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>cerebrovascular imaging;anticoagulation;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;anticoagulation;secondary prevention;cerebrovascular imaging</t>
         </is>
       </c>
       <c r="I484" t="n">
@@ -29134,7 +29134,7 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>secondary prevention;anticoagulation;ischemic stroke;TIA</t>
+          <t>ischemic stroke;anticoagulation;secondary prevention;TIA</t>
         </is>
       </c>
       <c r="I514" t="n">
@@ -29918,7 +29918,7 @@
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke;antiplatelet therapy</t>
+          <t>ischemic stroke;secondary prevention;antiplatelet therapy</t>
         </is>
       </c>
       <c r="I528" t="n">
@@ -32630,7 +32630,7 @@
       </c>
       <c r="H577" t="inlineStr">
         <is>
-          <t>carotid stenosis;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;carotid stenosis;secondary prevention</t>
         </is>
       </c>
       <c r="I577" t="n">
@@ -35306,7 +35306,7 @@
       </c>
       <c r="H624" t="inlineStr">
         <is>
-          <t>secondary prevention;stroke rehabilitation;ischemic stroke;endovascular thrombectomy</t>
+          <t>ischemic stroke;stroke rehabilitation;secondary prevention;endovascular thrombectomy</t>
         </is>
       </c>
       <c r="I624" t="n">
@@ -37634,7 +37634,7 @@
       </c>
       <c r="H666" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke;endovascular thrombectomy</t>
+          <t>ischemic stroke;secondary prevention;endovascular thrombectomy</t>
         </is>
       </c>
       <c r="I666" t="n">
@@ -39006,7 +39006,7 @@
       </c>
       <c r="H690" t="inlineStr">
         <is>
-          <t>stroke rehabilitation;cerebrovascular imaging;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;stroke rehabilitation;secondary prevention;cerebrovascular imaging</t>
         </is>
       </c>
       <c r="I690" t="n">
@@ -42302,7 +42302,7 @@
       </c>
       <c r="H749" t="inlineStr">
         <is>
-          <t>secondary prevention;lipid management;atrial fibrillation;ischemic stroke</t>
+          <t>ischemic stroke;secondary prevention;atrial fibrillation;lipid management</t>
         </is>
       </c>
       <c r="I749" t="n">
@@ -42754,7 +42754,7 @@
       </c>
       <c r="H757" t="inlineStr">
         <is>
-          <t>lipid management;secondary prevention;TIA;ischemic stroke</t>
+          <t>ischemic stroke;secondary prevention;lipid management;TIA</t>
         </is>
       </c>
       <c r="I757" t="n">
@@ -45026,7 +45026,7 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>antiplatelet therapy;secondary prevention;ischemic stroke;telestroke;TIA</t>
+          <t>ischemic stroke;TIA;telestroke;secondary prevention;antiplatelet therapy</t>
         </is>
       </c>
       <c r="I798" t="n">
@@ -46010,7 +46010,7 @@
       </c>
       <c r="H816" t="inlineStr">
         <is>
-          <t>lipid management;secondary prevention;ischemic stroke;telestroke;anticoagulation</t>
+          <t>ischemic stroke;telestroke;anticoagulation;secondary prevention;lipid management</t>
         </is>
       </c>
       <c r="I816" t="n">
@@ -48378,7 +48378,7 @@
       </c>
       <c r="H858" t="inlineStr">
         <is>
-          <t>TIA;anticoagulation;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;anticoagulation;secondary prevention;TIA</t>
         </is>
       </c>
       <c r="I858" t="n">
@@ -49154,7 +49154,7 @@
       </c>
       <c r="H872" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;secondary prevention</t>
         </is>
       </c>
       <c r="I872" t="n">
@@ -49434,7 +49434,7 @@
       </c>
       <c r="H877" t="inlineStr">
         <is>
-          <t>carotid stenosis;secondary prevention;ischemic stroke;antiplatelet therapy</t>
+          <t>ischemic stroke;carotid stenosis;secondary prevention;antiplatelet therapy</t>
         </is>
       </c>
       <c r="I877" t="n">
@@ -51482,7 +51482,7 @@
       </c>
       <c r="H914" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke;telestroke</t>
+          <t>ischemic stroke;telestroke;secondary prevention</t>
         </is>
       </c>
       <c r="I914" t="n">
@@ -53218,7 +53218,7 @@
       </c>
       <c r="H945" t="inlineStr">
         <is>
-          <t>stroke rehabilitation;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;stroke rehabilitation;secondary prevention</t>
         </is>
       </c>
       <c r="I945" t="n">
@@ -64294,7 +64294,7 @@
       </c>
       <c r="H1143" t="inlineStr">
         <is>
-          <t>secondary prevention;stroke rehabilitation;ischemic stroke;TIA</t>
+          <t>ischemic stroke;stroke rehabilitation;secondary prevention;TIA</t>
         </is>
       </c>
       <c r="I1143" t="n">
@@ -64794,7 +64794,7 @@
       </c>
       <c r="H1152" t="inlineStr">
         <is>
-          <t>lipid management;endovascular thrombectomy;secondary prevention;telestroke;ischemic stroke</t>
+          <t>ischemic stroke;telestroke;secondary prevention;lipid management;endovascular thrombectomy</t>
         </is>
       </c>
       <c r="I1152" t="n">
@@ -65146,7 +65146,7 @@
       </c>
       <c r="H1158" t="inlineStr">
         <is>
-          <t>cerebrovascular imaging;secondary prevention;ischemic stroke;antiplatelet therapy</t>
+          <t>ischemic stroke;secondary prevention;antiplatelet therapy;cerebrovascular imaging</t>
         </is>
       </c>
       <c r="I1158" t="n">
@@ -71690,7 +71690,7 @@
       </c>
       <c r="H1275" t="inlineStr">
         <is>
-          <t>lipid management;secondary prevention;ischemic stroke;anticoagulation;atrial fibrillation</t>
+          <t>ischemic stroke;anticoagulation;secondary prevention;lipid management;atrial fibrillation</t>
         </is>
       </c>
       <c r="I1275" t="n">
@@ -76062,7 +76062,7 @@
       </c>
       <c r="H1353" t="inlineStr">
         <is>
-          <t>anticoagulation;secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;anticoagulation;secondary prevention</t>
         </is>
       </c>
       <c r="I1353" t="n">
@@ -77958,7 +77958,7 @@
       </c>
       <c r="H1387" t="inlineStr">
         <is>
-          <t>secondary prevention;ischemic stroke</t>
+          <t>ischemic stroke;secondary prevention</t>
         </is>
       </c>
       <c r="I1387" t="n">

</xml_diff>